<commit_message>
Ex3A tables and script
</commit_message>
<xml_diff>
--- a/Ruiz_Ex3A_tables.xlsx
+++ b/Ruiz_Ex3A_tables.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/04a19e4a9bb9275a/Documents/DATA_Labs/W2_Workshop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="56" documentId="11_F25DC773A252ABDACC1048C6311C79EA5ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7A4DE494-F370-4502-AFB0-D0534563E2B4}"/>
+  <xr:revisionPtr revIDLastSave="68" documentId="11_F25DC773A252ABDACC1048C6311C79EA5ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{20241DAC-A1C3-4DFA-8FFA-CA2012813B21}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13056" firstSheet="2" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="8748" windowHeight="13056" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Customer" sheetId="1" r:id="rId1"/>
@@ -29,26 +29,11 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="24">
-  <si>
-    <t>FirstName</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="28">
   <si>
     <t>CustomerID</t>
   </si>
   <si>
-    <t>LastName</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>Phone</t>
-  </si>
-  <si>
-    <t>Address</t>
-  </si>
-  <si>
     <t>DogID</t>
   </si>
   <si>
@@ -101,6 +86,33 @@
   </si>
   <si>
     <t>Notes</t>
+  </si>
+  <si>
+    <t>CustomerFirstName</t>
+  </si>
+  <si>
+    <t>CustomerLastName</t>
+  </si>
+  <si>
+    <t>CustomerEmail</t>
+  </si>
+  <si>
+    <t>CustomerPhone</t>
+  </si>
+  <si>
+    <t>CustomerAddress</t>
+  </si>
+  <si>
+    <t>WalkerFirstName</t>
+  </si>
+  <si>
+    <t>WalkerLastName</t>
+  </si>
+  <si>
+    <t>WalkerEmail</t>
+  </si>
+  <si>
+    <t>WalkerPhone</t>
   </si>
 </sst>
 </file>
@@ -167,6 +179,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -434,25 +450,33 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="B2:G2"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="17.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.33203125" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C2" t="s">
-        <v>0</v>
+        <v>19</v>
       </c>
       <c r="D2" t="s">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="E2" t="s">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="F2" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="G2" t="s">
-        <v>5</v>
+        <v>23</v>
       </c>
     </row>
   </sheetData>
@@ -476,25 +500,25 @@
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H2" t="s">
         <v>6</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" t="s">
-        <v>10</v>
-      </c>
-      <c r="H2" t="s">
-        <v>11</v>
       </c>
     </row>
   </sheetData>
@@ -508,31 +532,31 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="9.33203125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="6.109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.109375" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.88671875" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="8.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
-        <v>12</v>
+        <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="D2" t="s">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="E2" t="s">
-        <v>3</v>
+        <v>26</v>
       </c>
       <c r="F2" t="s">
-        <v>4</v>
+        <v>27</v>
       </c>
       <c r="G2" t="s">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -556,25 +580,25 @@
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>10</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="E2" t="s">
+        <v>11</v>
+      </c>
+      <c r="F2" t="s">
+        <v>12</v>
+      </c>
+      <c r="G2" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" t="s">
         <v>14</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" t="s">
-        <v>16</v>
-      </c>
-      <c r="F2" t="s">
-        <v>17</v>
-      </c>
-      <c r="G2" t="s">
-        <v>18</v>
-      </c>
-      <c r="H2" t="s">
-        <v>19</v>
       </c>
     </row>
   </sheetData>
@@ -597,25 +621,25 @@
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.3">
       <c r="B2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
         <v>15</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E2" t="s">
-        <v>20</v>
-      </c>
       <c r="F2" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="G2" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="H2" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Updated Ex3A for Ex4A module
</commit_message>
<xml_diff>
--- a/Ruiz_Ex3A_tables.xlsx
+++ b/Ruiz_Ex3A_tables.xlsx
@@ -8,16 +8,16 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/04a19e4a9bb9275a/Documents/DATA_Labs/W2_Workshop/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="68" documentId="11_F25DC773A252ABDACC1048C6311C79EA5ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{20241DAC-A1C3-4DFA-8FFA-CA2012813B21}"/>
+  <xr:revisionPtr revIDLastSave="113" documentId="11_F25DC773A252ABDACC1048C6311C79EA5ADE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1FF89BE7-C25B-4534-B0C8-6DA9A419C042}"/>
   <bookViews>
-    <workbookView xWindow="-96" yWindow="0" windowWidth="8748" windowHeight="13056" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-96" yWindow="0" windowWidth="11712" windowHeight="13056" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Customer" sheetId="1" r:id="rId1"/>
     <sheet name="Dogs" sheetId="2" r:id="rId2"/>
     <sheet name="Walkers" sheetId="3" r:id="rId3"/>
-    <sheet name="Transactions" sheetId="4" r:id="rId4"/>
-    <sheet name="Walks" sheetId="5" r:id="rId5"/>
+    <sheet name="Walks" sheetId="5" r:id="rId4"/>
+    <sheet name="Transactions" sheetId="4" r:id="rId5"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -29,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="28">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="49" uniqueCount="44">
   <si>
     <t>CustomerID</t>
   </si>
@@ -113,16 +113,72 @@
   </si>
   <si>
     <t>WalkerPhone</t>
+  </si>
+  <si>
+    <t>Maria</t>
+  </si>
+  <si>
+    <t>Cervantes</t>
+  </si>
+  <si>
+    <t>mcervantes@gmail.com</t>
+  </si>
+  <si>
+    <t>4552 Sesame Street Chicago, IL 65879</t>
+  </si>
+  <si>
+    <t>Vicky</t>
+  </si>
+  <si>
+    <t>Pitbull</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>3 years</t>
+  </si>
+  <si>
+    <t>Scared of cars honking</t>
+  </si>
+  <si>
+    <t>Martha</t>
+  </si>
+  <si>
+    <t>Nunez</t>
+  </si>
+  <si>
+    <t>mnunez@gmail.com</t>
+  </si>
+  <si>
+    <t>45 minutes</t>
+  </si>
+  <si>
+    <t>First walk of the day</t>
+  </si>
+  <si>
+    <t>VISA</t>
+  </si>
+  <si>
+    <t>Approved</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -157,15 +213,20 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="21" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -448,15 +509,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:G2"/>
+  <dimension ref="B2:G3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="17.44140625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="17.33203125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="13.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="14.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="18.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.88671875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="22.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="14.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="34.5546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.3">
@@ -479,64 +540,110 @@
         <v>23</v>
       </c>
     </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" t="s">
+        <v>29</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3">
+        <v>7734447789</v>
+      </c>
+      <c r="G3" t="s">
+        <v>31</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E3" r:id="rId1" xr:uid="{68408CAF-F156-40C2-A36F-B8B7DC7AA964}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CE7DF9C-A4F3-41B3-8E61-F7C6A49506EA}">
+  <dimension ref="B2:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="6.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.21875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="7.44140625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.21875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" t="s">
+        <v>2</v>
+      </c>
+      <c r="E2" t="s">
+        <v>3</v>
+      </c>
+      <c r="F2" t="s">
+        <v>4</v>
+      </c>
+      <c r="G2" t="s">
+        <v>5</v>
+      </c>
+      <c r="H2" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" t="s">
+        <v>33</v>
+      </c>
+      <c r="F3" t="s">
+        <v>34</v>
+      </c>
+      <c r="G3" t="s">
+        <v>35</v>
+      </c>
+      <c r="H3" t="s">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CE7DF9C-A4F3-41B3-8E61-F7C6A49506EA}">
-  <dimension ref="B2:H2"/>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39EA9141-0F89-4364-86D4-867267E9CC58}">
+  <dimension ref="B2:G3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="6" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="9.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="5.77734375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="4.109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="4" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="11.5546875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>0</v>
-      </c>
-      <c r="D2" t="s">
-        <v>2</v>
-      </c>
-      <c r="E2" t="s">
-        <v>3</v>
-      </c>
-      <c r="F2" t="s">
-        <v>4</v>
-      </c>
-      <c r="G2" t="s">
-        <v>5</v>
-      </c>
-      <c r="H2" t="s">
-        <v>6</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{39EA9141-0F89-4364-86D4-867267E9CC58}">
-  <dimension ref="B2:G2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.109375" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.21875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.88671875" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.44140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="18.88671875" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.77734375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:7" x14ac:dyDescent="0.3">
@@ -559,23 +666,110 @@
         <v>8</v>
       </c>
     </row>
+    <row r="3" spans="2:7" x14ac:dyDescent="0.3">
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D3" t="s">
+        <v>38</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="F3">
+        <v>3125478896</v>
+      </c>
+      <c r="G3" s="4">
+        <v>44958</v>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="E3" r:id="rId1" xr:uid="{FD51E3A2-CDD2-4AD3-9A6C-6090253713F5}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72C5A269-FF8F-4D79-BA63-D90A4E1F1000}">
+  <dimension ref="B2:H3"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="2" max="2" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="6.33203125" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="9.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.6640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18.88671875" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B2" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F2" t="s">
+        <v>16</v>
+      </c>
+      <c r="G2" t="s">
+        <v>17</v>
+      </c>
+      <c r="H2" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B3">
+        <v>1</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3" s="5">
+        <v>0.54305555555555551</v>
+      </c>
+      <c r="F3" s="5">
+        <v>0.57430555555555551</v>
+      </c>
+      <c r="G3" t="s">
+        <v>40</v>
+      </c>
+      <c r="H3" t="s">
+        <v>41</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BB9A2747-51F3-415A-B882-14C3BE0B4B38}">
-  <dimension ref="B2:H2"/>
+  <dimension ref="B2:H3"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="12.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="10.6640625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="7.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="14.6640625" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="13.44140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="7.5546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="7.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.44140625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.33203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.33203125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="2:8" x14ac:dyDescent="0.3">
@@ -601,45 +795,27 @@
         <v>14</v>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{72C5A269-FF8F-4D79-BA63-D90A4E1F1000}">
-  <dimension ref="B2:H2"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
-  <cols>
-    <col min="2" max="2" width="6.88671875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="6" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="8.5546875" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="8.109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="5.88671875" bestFit="1" customWidth="1"/>
-  </cols>
-  <sheetData>
-    <row r="2" spans="2:8" x14ac:dyDescent="0.3">
-      <c r="B2" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>1</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="E2" t="s">
-        <v>15</v>
-      </c>
-      <c r="F2" t="s">
-        <v>16</v>
-      </c>
-      <c r="G2" t="s">
-        <v>17</v>
-      </c>
-      <c r="H2" t="s">
-        <v>18</v>
+    <row r="3" spans="2:8" x14ac:dyDescent="0.3">
+      <c r="B3">
+        <v>62646741</v>
+      </c>
+      <c r="C3">
+        <v>1</v>
+      </c>
+      <c r="D3">
+        <v>1</v>
+      </c>
+      <c r="E3">
+        <v>50</v>
+      </c>
+      <c r="F3" s="4">
+        <v>46129</v>
+      </c>
+      <c r="G3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H3" t="s">
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>